<commit_message>
Actualizacion datos REM 2026-09-29 16:03 (orquestador)
</commit_message>
<xml_diff>
--- a/output/cobertura_mamografia_rm_2025.xlsx
+++ b/output/cobertura_mamografia_rm_2025.xlsx
@@ -2685,7 +2685,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Centro Comunitario de Salud Familiar Dr. José Symón Ojeda</t>
+          <t>CECOSF Haydeé Sepúlveda</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -6142,7 +6142,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>Hospital de Til Til</t>
+          <t>Hospital Comunitario de Til Til</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -11457,7 +11457,7 @@
       </c>
       <c r="W97" t="inlineStr">
         <is>
-          <t>Cerrado</t>
+          <t>Vigente en Operación Habitual</t>
         </is>
       </c>
       <c r="X97" t="b">
@@ -12220,7 +12220,7 @@
       </c>
       <c r="T105" t="inlineStr">
         <is>
-          <t>Centro Comunitario de Salud Familiar Lo Chacón</t>
+          <t>CECOSF Wilma Yoli Gomez Conejera</t>
         </is>
       </c>
       <c r="U105" t="inlineStr">
@@ -21622,7 +21622,7 @@
       </c>
       <c r="T202" t="inlineStr">
         <is>
-          <t>Centro de Salud Familiar Maipo</t>
+          <t>Centro de Salud Familiar Dragica Ciudad Pap</t>
         </is>
       </c>
       <c r="U202" t="inlineStr">
@@ -29987,7 +29987,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Centro Comunitario de Salud Familiar Dr. José Symón Ojeda</t>
+          <t>CECOSF Haydeé Sepúlveda</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -30612,7 +30612,7 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Centro de Referencia de Salud (CRS)</t>
+          <t>Centro de Especialidades</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
@@ -34172,7 +34172,7 @@
       </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t>Cerrado</t>
+          <t>Vigente en Operación Habitual</t>
         </is>
       </c>
     </row>
@@ -36537,7 +36537,7 @@
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>Centro de Referencia de Salud (CRS)</t>
+          <t>Centro de Especialidades</t>
         </is>
       </c>
       <c r="L120" t="inlineStr">
@@ -39817,7 +39817,7 @@
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>Centro de Referencia de Salud (CRS)</t>
+          <t>Centro de Especialidades</t>
         </is>
       </c>
       <c r="L163" t="inlineStr">
@@ -41397,7 +41397,7 @@
       </c>
       <c r="L184" t="inlineStr">
         <is>
-          <t>Centro de Salud Familiar Maipo</t>
+          <t>Centro de Salud Familiar Dragica Ciudad Pap</t>
         </is>
       </c>
       <c r="M184" t="inlineStr">
@@ -48967,7 +48967,7 @@
       </c>
       <c r="L283" t="inlineStr">
         <is>
-          <t>Centro Comunitario de Salud Familiar Lo Chacón</t>
+          <t>CECOSF Wilma Yoli Gomez Conejera</t>
         </is>
       </c>
       <c r="M283" t="inlineStr">
@@ -50028,7 +50028,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Hospital de Til Til</t>
+          <t>Hospital Comunitario de Til Til</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">

</xml_diff>